<commit_message>
Adicionado o teste de apontar ordem e modo simulado e modo real como foi solicitado
</commit_message>
<xml_diff>
--- a/data/input/Cenários de Testes Unitários e Parciais - PM-Manutenção  1.xlsx
+++ b/data/input/Cenários de Testes Unitários e Parciais - PM-Manutenção  1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juscelinob\Documents\automated-integrated-tests\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA853934-3955-4745-8D83-0255E7005534}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5499761-8071-4A9F-9D3D-87C904F5084B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="143">
   <si>
     <t>Status</t>
   </si>
@@ -335,106 +335,124 @@
     <t>IW28 - Criar Ordem de manutenção tipo "ZMEL" para a nota Z4.</t>
   </si>
   <si>
+    <t>Transação</t>
+  </si>
+  <si>
+    <t>UNIT_PM_WMO_01</t>
+  </si>
+  <si>
+    <t>IW21</t>
+  </si>
+  <si>
+    <t>Parametro</t>
+  </si>
+  <si>
+    <t>IW31</t>
+  </si>
+  <si>
+    <t>IW32</t>
+  </si>
+  <si>
+    <t>IW41</t>
+  </si>
+  <si>
+    <t>IP41</t>
+  </si>
+  <si>
+    <t>IP42</t>
+  </si>
+  <si>
+    <t>IW34</t>
+  </si>
+  <si>
+    <t>ME21N</t>
+  </si>
+  <si>
+    <t>MIGO</t>
+  </si>
+  <si>
+    <t>MIRO</t>
+  </si>
+  <si>
+    <t>F110</t>
+  </si>
+  <si>
+    <t>KO88</t>
+  </si>
+  <si>
+    <t>IW32 - Process to finish the order</t>
+  </si>
+  <si>
+    <t>IP10</t>
+  </si>
+  <si>
+    <t>MB26</t>
+  </si>
+  <si>
+    <t>IP30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SBWP </t>
+  </si>
+  <si>
+    <t>IW28</t>
+  </si>
+  <si>
+    <t>Criar Ordem Manutenção tipo ZCOR - IW31</t>
+  </si>
+  <si>
+    <t>UNIT_PM_WMO_02</t>
+  </si>
+  <si>
     <t>Criar Nota de Manutenção tipo Z1 - IW21</t>
   </si>
   <si>
-    <t>Transação</t>
-  </si>
-  <si>
-    <t>UNIT_PM_WMO_01</t>
-  </si>
-  <si>
-    <t>IW21</t>
-  </si>
-  <si>
-    <t>Parametro</t>
-  </si>
-  <si>
-    <t>IW31</t>
-  </si>
-  <si>
-    <t>IW32</t>
-  </si>
-  <si>
-    <t>IW41</t>
-  </si>
-  <si>
-    <t>IP41</t>
-  </si>
-  <si>
-    <t>IP42</t>
-  </si>
-  <si>
-    <t>IW34</t>
-  </si>
-  <si>
-    <t>ME21N</t>
-  </si>
-  <si>
-    <t>MIGO</t>
-  </si>
-  <si>
-    <t>MIRO</t>
-  </si>
-  <si>
-    <t>F110</t>
-  </si>
-  <si>
-    <t>KO88</t>
-  </si>
-  <si>
-    <t>IW32 - Process to finish the order</t>
-  </si>
-  <si>
-    <t>IP10</t>
-  </si>
-  <si>
-    <t>MB26</t>
-  </si>
-  <si>
-    <t>IP30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SBWP </t>
-  </si>
-  <si>
-    <t>IW28</t>
-  </si>
-  <si>
-    <t>UNIT_PM_WMO_02</t>
+    <t>LI: D10167100-S10167120 | Texto Breve: teste | Notificador: teste | Prioridade: 1 | Ramal: 1111</t>
   </si>
   <si>
     <t>UNIT_PM_WMO_03</t>
   </si>
   <si>
-    <t>Criar Ordem Manutenção tipo ZCOR - IW31</t>
+    <t>Criar Ordem Manutenção tipo ZMEL - IW31</t>
   </si>
   <si>
     <t>UNIT_PM_WMO_04</t>
   </si>
   <si>
-    <t>Criar Ordem Manutenção tipo ZMEL - IW31</t>
+    <t>Criar Ordem Manutenção tipo ZPRE - IW31</t>
+  </si>
+  <si>
+    <t>LI: D10167100-S10167120 | Texto Breve: testeO | TipoAtvMnt: 31 | Prioridade: 2 | Criar Nota: x | Notificador: teste | Prioridade da Nota: 1 | Ramal: 1111 | Trabalho: 1 | Nº Colaboradores: 1</t>
+  </si>
+  <si>
+    <t>Equipamento: 10141343 | Texto Breve: testeO | TipoAtvMnt: 19 | Prioridade: 3  | Criar Nota: x | Notificador: teste | Prioridade da Nota: 1 | Ramal: 1111 | Trabalho: 1 | Nº Colaboradores: 1</t>
+  </si>
+  <si>
+    <t>LI: D10167100-S10167120 | Texto Breve: testeO | TipoAtvMnt: 28 | Prioridade: 1 | Criar Nota: x | Notificador: teste | Prioridade da Nota: 1 | Ramal: 1111 | Trabalho: 1 | Nº Colaboradores: 1 | Texto Operação 2: teste2 | Trabalho 2: 1 | Nº colaboradores 2: 1</t>
+  </si>
+  <si>
+    <t>Imprimir Ordem Manutenção - IW32</t>
   </si>
   <si>
     <t>UNIT_PM_WMO_05</t>
   </si>
   <si>
-    <t>Criar Ordem Manutenção tipo ZPRE - IW31</t>
-  </si>
-  <si>
-    <t>Imprimir Ordem Manutenção - IW32</t>
-  </si>
-  <si>
-    <t>LI: D10167100-S10167120 | Texto Breve: teste | TipoAtvMnt: 28 | Prioridade : 1 | Trabalho: 1 | Nº Colaboradores: 1</t>
-  </si>
-  <si>
-    <t>LI: D10167100-S10167120 | Texto Breve: teste | TipoAtvMnt: 31 | Prioridade: 2 | Trabalho: 1 | Nº Colaboradores: 1</t>
-  </si>
-  <si>
-    <t>Equipamento: 10141343 | Texto Breve: teste | TipoAtvMnt: 19 | Prioridade: 3  | Trabalho: 1 | Nº Colaboradores: 1</t>
-  </si>
-  <si>
-    <t>LI: D10167100-S10167120  | Tipo de nota: Z1 | Texto Breve: teste | Notificador: teste | Prioridade: 1 | Ramal: 1111</t>
+    <t>UNIT_PM_WMO_07</t>
+  </si>
+  <si>
+    <t>Apontar Ordem Manutenção - IW41</t>
+  </si>
+  <si>
+    <t>Nº pessoal: 111027</t>
+  </si>
+  <si>
+    <t>Modo</t>
+  </si>
+  <si>
+    <t>simulado</t>
+  </si>
+  <si>
+    <t>real</t>
   </si>
 </sst>
 </file>
@@ -988,7 +1006,7 @@
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1011,15 +1029,20 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="13" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Ênfase1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1366,133 +1389,240 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9ADDAA96-011D-4AD4-8D95-F536D2754849}">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8.81640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.7265625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="37.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="98.36328125" customWidth="1"/>
-    <col min="6" max="6" width="7.6328125" customWidth="1"/>
+    <col min="5" max="5" width="255.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="28.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="F1" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1" s="17" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2" s="13">
+        <v>1</v>
+      </c>
+      <c r="B2" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="C2" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="C2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D2" t="s">
-        <v>103</v>
-      </c>
-      <c r="E2" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="D2" s="13" t="s">
+        <v>126</v>
+      </c>
+      <c r="E2" s="13" t="s">
+        <v>127</v>
+      </c>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="13">
         <v>1</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="13" t="s">
         <v>125</v>
       </c>
-      <c r="C3" s="14" t="s">
-        <v>108</v>
-      </c>
-      <c r="D3" s="14" t="s">
-        <v>127</v>
-      </c>
-      <c r="E3" s="14" t="s">
+      <c r="C3" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" s="13">
+        <v>1</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="F4" s="13"/>
+      <c r="G4" s="13" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" s="13">
+        <v>1</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>130</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="E5" s="13" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" s="15">
-        <v>1</v>
-      </c>
-      <c r="B4" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>108</v>
-      </c>
-      <c r="D4" s="14" t="s">
-        <v>129</v>
-      </c>
-      <c r="E4" s="14" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" s="15">
-        <v>1</v>
-      </c>
-      <c r="B5" s="14" t="s">
-        <v>128</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>108</v>
-      </c>
-      <c r="D5" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="E5" s="14" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="F5" s="13"/>
+      <c r="G5" s="13" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="13">
         <v>1</v>
       </c>
-      <c r="B6" s="14" t="s">
-        <v>130</v>
-      </c>
-      <c r="C6" s="14" t="s">
+      <c r="B6" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="E6" s="13"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="13" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>1</v>
+      </c>
+      <c r="B7" t="s">
+        <v>137</v>
+      </c>
+      <c r="C7" t="s">
         <v>109</v>
       </c>
-      <c r="D6" s="14" t="s">
-        <v>132</v>
-      </c>
-      <c r="E6" s="14"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7" s="13"/>
-      <c r="B7" s="14"/>
-      <c r="C7" s="14"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="D7" t="s">
+        <v>138</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" s="13"/>
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="13"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" s="13"/>
+      <c r="B9" s="13"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="13"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10" s="13"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="13"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11" s="13"/>
+      <c r="B11" s="13"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
       <c r="E11" s="16"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="13"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A12" s="13"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A13" s="13"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="13"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A14" s="13"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="13"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A15" s="13"/>
+      <c r="B15" s="13"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="13"/>
     </row>
   </sheetData>
   <phoneticPr fontId="20" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1527,7 +1657,7 @@
         <v>5</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>0</v>
@@ -1550,7 +1680,7 @@
         <v>34</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G2" s="5"/>
     </row>
@@ -1571,7 +1701,7 @@
         <v>36</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G3" s="5"/>
     </row>
@@ -1592,7 +1722,7 @@
         <v>38</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G4" s="3"/>
     </row>
@@ -1613,7 +1743,7 @@
         <v>40</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G5" s="5"/>
     </row>
@@ -1653,7 +1783,7 @@
         <v>42</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G7" s="3"/>
     </row>
@@ -1674,7 +1804,7 @@
         <v>44</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G8" s="5"/>
     </row>
@@ -1695,7 +1825,7 @@
         <v>46</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G9" s="3"/>
     </row>
@@ -1716,7 +1846,7 @@
         <v>48</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G10" s="5"/>
     </row>
@@ -1737,7 +1867,7 @@
         <v>50</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G11" s="3"/>
     </row>
@@ -1758,7 +1888,7 @@
         <v>52</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G12" s="5"/>
     </row>
@@ -1779,7 +1909,7 @@
         <v>54</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G13" s="3"/>
     </row>
@@ -1800,7 +1930,7 @@
         <v>34</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G14" s="5"/>
     </row>
@@ -1821,7 +1951,7 @@
         <v>36</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G15" s="5"/>
     </row>
@@ -1842,7 +1972,7 @@
         <v>20</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G16" s="5"/>
     </row>
@@ -1863,7 +1993,7 @@
         <v>8</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G17" s="3"/>
     </row>
@@ -1884,7 +2014,7 @@
         <v>10</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G18" s="5"/>
     </row>
@@ -1905,7 +2035,7 @@
         <v>12</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G19" s="3"/>
     </row>
@@ -1926,7 +2056,7 @@
         <v>14</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G20" s="5"/>
     </row>
@@ -1944,10 +2074,10 @@
         <v>15</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G21" s="3"/>
     </row>
@@ -1968,7 +2098,7 @@
         <v>17</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G22" s="5"/>
     </row>
@@ -1989,7 +2119,7 @@
         <v>86</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G23" s="3"/>
     </row>
@@ -2010,7 +2140,7 @@
         <v>88</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G24" s="5"/>
     </row>
@@ -2031,7 +2161,7 @@
         <v>38</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G25" s="3"/>
     </row>
@@ -2052,7 +2182,7 @@
         <v>90</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G26" s="5"/>
     </row>
@@ -2073,7 +2203,7 @@
         <v>68</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G27" s="3"/>
     </row>
@@ -2094,7 +2224,7 @@
         <v>50</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G28" s="5"/>
     </row>
@@ -2115,7 +2245,7 @@
         <v>52</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G29" s="3"/>
     </row>
@@ -2136,7 +2266,7 @@
         <v>54</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G30" s="5"/>
     </row>
@@ -2157,7 +2287,7 @@
         <v>92</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G31" s="3"/>
     </row>
@@ -2178,7 +2308,7 @@
         <v>94</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G32" s="5"/>
     </row>
@@ -2199,7 +2329,7 @@
         <v>95</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G33" s="3"/>
     </row>
@@ -2220,7 +2350,7 @@
         <v>38</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G34" s="5"/>
     </row>
@@ -2241,7 +2371,7 @@
         <v>96</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G35" s="3"/>
     </row>
@@ -2262,7 +2392,7 @@
         <v>52</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G36" s="5"/>
     </row>
@@ -2283,7 +2413,7 @@
         <v>54</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G37" s="3"/>
     </row>
@@ -2323,7 +2453,7 @@
         <v>99</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G39" s="5"/>
     </row>
@@ -2344,7 +2474,7 @@
         <v>101</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G40" s="3"/>
     </row>
@@ -2365,7 +2495,7 @@
         <v>102</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G41" s="5"/>
     </row>
@@ -2386,7 +2516,7 @@
         <v>38</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G42" s="3"/>
     </row>
@@ -2407,7 +2537,7 @@
         <v>90</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G43" s="5"/>
     </row>
@@ -2428,7 +2558,7 @@
         <v>68</v>
       </c>
       <c r="F44" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G44" s="3"/>
     </row>
@@ -2449,7 +2579,7 @@
         <v>96</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G45" s="5"/>
     </row>
@@ -2470,7 +2600,7 @@
         <v>52</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G46" s="3"/>
     </row>
@@ -2491,7 +2621,7 @@
         <v>54</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G47" s="5"/>
     </row>
@@ -2550,7 +2680,7 @@
         <v>62</v>
       </c>
       <c r="F50" s="12" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G50" s="3"/>
     </row>
@@ -2571,7 +2701,7 @@
         <v>64</v>
       </c>
       <c r="F51" s="11" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G51" s="5"/>
     </row>
@@ -2611,7 +2741,7 @@
         <v>68</v>
       </c>
       <c r="F53" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G53" s="3"/>
     </row>
@@ -2632,7 +2762,7 @@
         <v>69</v>
       </c>
       <c r="F54" s="12" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G54" s="5"/>
     </row>
@@ -2653,7 +2783,7 @@
         <v>71</v>
       </c>
       <c r="F55" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G55" s="3"/>
     </row>
@@ -2674,7 +2804,7 @@
         <v>73</v>
       </c>
       <c r="F56" s="12" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G56" s="5"/>
     </row>
@@ -2695,7 +2825,7 @@
         <v>74</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G57" s="3"/>
     </row>
@@ -2716,7 +2846,7 @@
         <v>76</v>
       </c>
       <c r="F58" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G58" s="5"/>
     </row>
@@ -2737,7 +2867,7 @@
         <v>78</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G59" s="3"/>
     </row>
@@ -2758,7 +2888,7 @@
         <v>80</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G60" s="5"/>
     </row>
@@ -2817,7 +2947,7 @@
         <v>34</v>
       </c>
       <c r="F63" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G63" s="3"/>
     </row>
@@ -2838,7 +2968,7 @@
         <v>36</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G64" s="5"/>
     </row>
@@ -2859,7 +2989,7 @@
         <v>64</v>
       </c>
       <c r="F65" s="11" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G65" s="3"/>
     </row>
@@ -2895,7 +3025,7 @@
         <v>68</v>
       </c>
       <c r="F67" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G67" s="5"/>
     </row>
@@ -2916,7 +3046,7 @@
         <v>69</v>
       </c>
       <c r="F68" s="12" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G68" s="3"/>
     </row>
@@ -2937,7 +3067,7 @@
         <v>71</v>
       </c>
       <c r="F69" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G69" s="5"/>
     </row>
@@ -2958,7 +3088,7 @@
         <v>73</v>
       </c>
       <c r="F70" s="12" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G70" s="3"/>
     </row>
@@ -2979,7 +3109,7 @@
         <v>74</v>
       </c>
       <c r="F71" s="11" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G71" s="5"/>
     </row>
@@ -3000,7 +3130,7 @@
         <v>76</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G72" s="5"/>
     </row>
@@ -3021,7 +3151,7 @@
         <v>78</v>
       </c>
       <c r="F73" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G73" s="5"/>
     </row>
@@ -3042,7 +3172,7 @@
         <v>80</v>
       </c>
       <c r="F74" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G74" s="3"/>
     </row>

</xml_diff>

<commit_message>
Resolvido problema da impressão salvando no modo simulado
</commit_message>
<xml_diff>
--- a/data/input/Cenários de Testes Unitários e Parciais - PM-Manutenção  1.xlsx
+++ b/data/input/Cenários de Testes Unitários e Parciais - PM-Manutenção  1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juscelinob\Documents\automated-integrated-tests\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5499761-8071-4A9F-9D3D-87C904F5084B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F348E8D-D8CE-4EB4-BE2F-71C3B712AC0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1006,7 +1006,7 @@
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1040,8 +1040,11 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
@@ -1504,7 +1507,7 @@
       </c>
       <c r="F5" s="13"/>
       <c r="G5" s="13" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
@@ -1523,11 +1526,11 @@
       <c r="E6" s="13"/>
       <c r="F6" s="13"/>
       <c r="G6" s="13" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7">
+      <c r="A7" s="18">
         <v>1</v>
       </c>
       <c r="B7" t="s">
@@ -1544,7 +1547,7 @@
       </c>
       <c r="F7" s="13"/>
       <c r="G7" s="13" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
adicionando os testes de criar nota z4 e ordem para as notas z4 pela transação IW34
</commit_message>
<xml_diff>
--- a/data/input/Cenários de Testes Unitários e Parciais - PM-Manutenção  1.xlsx
+++ b/data/input/Cenários de Testes Unitários e Parciais - PM-Manutenção  1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juscelinob\Documents\automated-integrated-tests\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA853934-3955-4745-8D83-0255E7005534}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1A27957-B953-41C9-8264-8B41ADB724B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="147">
   <si>
     <t>Status</t>
   </si>
@@ -435,6 +435,36 @@
   </si>
   <si>
     <t>LI: D10167100-S10167120  | Tipo de nota: Z1 | Texto Breve: teste | Notificador: teste | Prioridade: 1 | Ramal: 1111</t>
+  </si>
+  <si>
+    <t>Criar Nota de Manutenção tipo Z4 - IW21</t>
+  </si>
+  <si>
+    <t>LI: D10167100-S10167120 | Tipo de nota: Z4 | Texto Breve: teste | Notificador: teste | Prioridade: 1 | Ramal: 1111</t>
+  </si>
+  <si>
+    <t>UNIT_PM_WMO_07</t>
+  </si>
+  <si>
+    <t>Apontar Ordem Manutenção - IW41</t>
+  </si>
+  <si>
+    <t>Nº pessoal: 111027</t>
+  </si>
+  <si>
+    <t>Criar Ordem Manutenção tipo ZMEL - IW34</t>
+  </si>
+  <si>
+    <t>LI: D10167100-S10167120 | Texto Breve: testeO | TipoAtvMnt: 31 | Prioridade: 2 | Criar Nota: x | Notificador: teste | Prioridade da Nota: 1 | Ramal: 1111 | Trabalho: 1 | Nº Colaboradores: 1</t>
+  </si>
+  <si>
+    <t>Modo</t>
+  </si>
+  <si>
+    <t>real</t>
+  </si>
+  <si>
+    <t>simulado</t>
   </si>
 </sst>
 </file>
@@ -988,7 +1018,7 @@
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1020,6 +1050,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Ênfase1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1366,18 +1397,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9ADDAA96-011D-4AD4-8D95-F536D2754849}">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8.81640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.7265625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="37.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="98.36328125" customWidth="1"/>
+    <col min="5" max="5" width="160.26953125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
         <v>1</v>
       </c>
@@ -1396,8 +1427,11 @@
       <c r="F1" s="1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G1" s="17" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1413,8 +1447,11 @@
       <c r="E2" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="13">
         <v>1</v>
       </c>
@@ -1430,8 +1467,11 @@
       <c r="E3" s="14" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G3" s="14" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="15">
         <v>1</v>
       </c>
@@ -1447,8 +1487,11 @@
       <c r="E4" s="14" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G4" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="15">
         <v>1</v>
       </c>
@@ -1464,8 +1507,11 @@
       <c r="E5" s="14" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G5" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="13">
         <v>1</v>
       </c>
@@ -1479,15 +1525,71 @@
         <v>132</v>
       </c>
       <c r="E6" s="14"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7" s="13"/>
-      <c r="B7" s="14"/>
-      <c r="C7" s="14"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G6" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" s="13">
+        <v>1</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="G7" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>1</v>
+      </c>
+      <c r="B8" t="s">
+        <v>139</v>
+      </c>
+      <c r="C8" t="s">
+        <v>110</v>
+      </c>
+      <c r="D8" t="s">
+        <v>140</v>
+      </c>
+      <c r="E8" t="s">
+        <v>141</v>
+      </c>
+      <c r="G8" s="14" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>1</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="G9" s="14" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="E11" s="16"/>
     </row>
   </sheetData>

</xml_diff>